<commit_message>
Corrida | SFE-ID | 2026-03-09 09:13:52.961583
</commit_message>
<xml_diff>
--- a/indicadores/SFE-ID_out.xlsx
+++ b/indicadores/SFE-ID_out.xlsx
@@ -106,13 +106,13 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">04/03/2026</t>
+    <t xml:space="preserve">09/03/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
   </si>
   <si>
-    <t xml:space="preserve">arodriguez</t>
+    <t xml:space="preserve">focampo</t>
   </si>
   <si>
     <t xml:space="preserve">fecha</t>

</xml_diff>

<commit_message>
Corrida | SFE-ID | 2026-03-10 10:10:43.043933
</commit_message>
<xml_diff>
--- a/indicadores/SFE-ID_out.xlsx
+++ b/indicadores/SFE-ID_out.xlsx
@@ -8,13 +8,14 @@
   <sheets>
     <sheet name="Portada" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Data" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Correlograma" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Referencias" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Correlograma" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="487" uniqueCount="487">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="509" uniqueCount="509">
   <si>
     <t xml:space="preserve"/>
   </si>
@@ -106,13 +107,13 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">09/03/2026</t>
+    <t xml:space="preserve">10/03/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
   </si>
   <si>
-    <t xml:space="preserve">pcohan</t>
+    <t xml:space="preserve">focampo</t>
   </si>
   <si>
     <t xml:space="preserve">fecha</t>
@@ -1412,6 +1413,72 @@
   </si>
   <si>
     <t xml:space="preserve">2030.12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Referencias.a.columnas.incluidas.en.la.hoja.DATA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">X2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Columna</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Descripcion</t>
+  </si>
+  <si>
+    <t xml:space="preserve">serie de datos brutos transformados, se importa directo desde base de datos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">a_original_fct_normal | serie original con 12 forecasts obtenidos del mejor modelo ARIMA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">a_original_fct_optimista | serie original con 12 forecasts, intervalo y límite optimista</t>
+  </si>
+  <si>
+    <t xml:space="preserve">a_original_fct_pesimista | serie original con 12 forecasts, intervalo y límite pesimista</t>
+  </si>
+  <si>
+    <t xml:space="preserve">b_d16 | salida D16 del X13-ARIMA-SEATS con los factores estacionales de la serie</t>
+  </si>
+  <si>
+    <t xml:space="preserve">c_c17 | salida C17 del X13-ARIMA-SEATS con pesos del irregular</t>
+  </si>
+  <si>
+    <t xml:space="preserve">d_d12 | salida D12 del X13-ARIMA-SEATS con el componente tendencia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">d_hp_129600 | tendencia HP de largo plazo con un lambda de 129.600</t>
+  </si>
+  <si>
+    <t xml:space="preserve">d_hp_200 | suavizado con filtro HP usando lambda de 200, sirve para determinar PG automáticos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">e_ajustada | serie ajustada por estacionalidad usando el mejor modelo (LOG o NIV según el caso)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">f_filtrada | serie ajustada por estacionalidad y corregida por irregularidad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">g_final | serie f_filtrada con o sin suavizado 2x2 según el caso (es la vieja española)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">g_final_fct_normal | a_original_fct ajustada por D16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gg_final_tcml | tasas de cambio mensual logarítmicas de la serie g_final</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gg_var_interanual | variaciones interanuales de g_final</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gg_final_var_mensual | variaciones mensuales de g_final</t>
+  </si>
+  <si>
+    <t xml:space="preserve">h_irregular | g_final/d_d12 componente irregular</t>
+  </si>
+  <si>
+    <t xml:space="preserve">i_dt | g_final/d_hp_129600 desvíos respecto de la tendencia</t>
   </si>
   <si>
     <t xml:space="preserve">Coeficientes de correlación de TCML del ICA-SFE y serie específica</t>
@@ -24744,203 +24811,573 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>0</v>
+        <v>466</v>
+      </c>
+      <c r="B1" t="s">
+        <v>467</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>466</v>
-      </c>
-      <c r="B2" s="1"/>
+        <v>468</v>
+      </c>
+      <c r="B2" t="s">
+        <v>469</v>
+      </c>
     </row>
     <row r="3">
-      <c r="A3"/>
-      <c r="B3" s="1"/>
+      <c r="A3" t="s">
+        <v>34</v>
+      </c>
+      <c r="B3" t="s">
+        <v>470</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>467</v>
-      </c>
-      <c r="B4" s="1"/>
+        <v>471</v>
+      </c>
+      <c r="B4"/>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>468</v>
-      </c>
-      <c r="B5" s="1" t="n">
-        <v>0.00901068154304649</v>
-      </c>
+        <v>472</v>
+      </c>
+      <c r="B5"/>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>469</v>
-      </c>
-      <c r="B6" s="1" t="n">
-        <v>0.0402007093603286</v>
-      </c>
+        <v>473</v>
+      </c>
+      <c r="B6"/>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>470</v>
-      </c>
-      <c r="B7" s="1" t="n">
-        <v>0.0845682923362035</v>
-      </c>
+        <v>474</v>
+      </c>
+      <c r="B7"/>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>471</v>
-      </c>
-      <c r="B8" s="1" t="n">
-        <v>0.161343160115743</v>
-      </c>
+        <v>475</v>
+      </c>
+      <c r="B8"/>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>472</v>
-      </c>
-      <c r="B9" s="1" t="n">
-        <v>0.220951473411767</v>
-      </c>
+        <v>476</v>
+      </c>
+      <c r="B9"/>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>473</v>
-      </c>
-      <c r="B10" s="1" t="n">
-        <v>0.292950805591597</v>
-      </c>
+        <v>477</v>
+      </c>
+      <c r="B10"/>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>474</v>
-      </c>
-      <c r="B11" s="1" t="n">
-        <v>0.380874935017229</v>
-      </c>
+        <v>478</v>
+      </c>
+      <c r="B11"/>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>475</v>
-      </c>
-      <c r="B12" s="1" t="n">
-        <v>0.451327417048397</v>
-      </c>
+        <v>479</v>
+      </c>
+      <c r="B12"/>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>476</v>
-      </c>
-      <c r="B13" s="1" t="n">
-        <v>0.517371477556427</v>
-      </c>
+        <v>480</v>
+      </c>
+      <c r="B13"/>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>477</v>
-      </c>
-      <c r="B14" s="1" t="n">
-        <v>0.617672515674822</v>
-      </c>
+        <v>481</v>
+      </c>
+      <c r="B14"/>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>478</v>
-      </c>
-      <c r="B15" s="1" t="n">
-        <v>0.595737749208721</v>
-      </c>
+        <v>482</v>
+      </c>
+      <c r="B15"/>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>479</v>
-      </c>
-      <c r="B16" s="1" t="n">
-        <v>0.578574411724506</v>
-      </c>
+        <v>483</v>
+      </c>
+      <c r="B16"/>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>480</v>
-      </c>
-      <c r="B17" s="1" t="n">
-        <v>0.565259695889537</v>
-      </c>
+        <v>484</v>
+      </c>
+      <c r="B17"/>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>481</v>
-      </c>
-      <c r="B18" s="1" t="n">
-        <v>0.53004013445323</v>
-      </c>
+        <v>485</v>
+      </c>
+      <c r="B18"/>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>482</v>
-      </c>
-      <c r="B19" s="1" t="n">
-        <v>0.535156403669814</v>
-      </c>
+        <v>486</v>
+      </c>
+      <c r="B19"/>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>483</v>
-      </c>
-      <c r="B20" s="1" t="n">
-        <v>0.475966041991827</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="s">
-        <v>484</v>
-      </c>
-      <c r="B21" s="1" t="n">
-        <v>0.388617541773781</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="s">
-        <v>485</v>
-      </c>
-      <c r="B22" s="1" t="n">
-        <v>0.340027575486936</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="s">
-        <v>486</v>
-      </c>
-      <c r="B23" s="1" t="n">
-        <v>0.312913062532667</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="B24" s="1"/>
-    </row>
-    <row r="25">
-      <c r="B25" s="1"/>
-    </row>
-    <row r="26">
-      <c r="B26" s="1"/>
-    </row>
-    <row r="27">
-      <c r="B27" s="1"/>
-    </row>
-    <row r="28">
-      <c r="B28" s="1"/>
-    </row>
-    <row r="29">
-      <c r="B29" s="1"/>
-    </row>
-    <row r="30">
-      <c r="B30" s="1"/>
+        <v>487</v>
+      </c>
+      <c r="B20"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>488</v>
+      </c>
+      <c r="B2" s="1"/>
+    </row>
+    <row r="3">
+      <c r="A3"/>
+      <c r="B3" s="1"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>489</v>
+      </c>
+      <c r="B4" s="1"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>490</v>
+      </c>
+      <c r="B5" s="1" t="n">
+        <v>0.00901068154304649</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>491</v>
+      </c>
+      <c r="B6" s="1" t="n">
+        <v>0.0402007093603286</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>492</v>
+      </c>
+      <c r="B7" s="1" t="n">
+        <v>0.0845682923362035</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>493</v>
+      </c>
+      <c r="B8" s="1" t="n">
+        <v>0.161343160115743</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>494</v>
+      </c>
+      <c r="B9" s="1" t="n">
+        <v>0.220951473411767</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>495</v>
+      </c>
+      <c r="B10" s="1" t="n">
+        <v>0.292950805591597</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>496</v>
+      </c>
+      <c r="B11" s="1" t="n">
+        <v>0.380874935017229</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>497</v>
+      </c>
+      <c r="B12" s="1" t="n">
+        <v>0.451327417048397</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s">
+        <v>498</v>
+      </c>
+      <c r="B13" s="1" t="n">
+        <v>0.517371477556427</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s">
+        <v>499</v>
+      </c>
+      <c r="B14" s="1" t="n">
+        <v>0.617672515674822</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s">
+        <v>500</v>
+      </c>
+      <c r="B15" s="1" t="n">
+        <v>0.595737749208721</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s">
+        <v>501</v>
+      </c>
+      <c r="B16" s="1" t="n">
+        <v>0.578574411724506</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s">
+        <v>502</v>
+      </c>
+      <c r="B17" s="1" t="n">
+        <v>0.565259695889537</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s">
+        <v>503</v>
+      </c>
+      <c r="B18" s="1" t="n">
+        <v>0.53004013445323</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s">
+        <v>504</v>
+      </c>
+      <c r="B19" s="1" t="n">
+        <v>0.535156403669814</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="s">
+        <v>505</v>
+      </c>
+      <c r="B20" s="1" t="n">
+        <v>0.475966041991827</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="s">
+        <v>506</v>
+      </c>
+      <c r="B21" s="1" t="n">
+        <v>0.388617541773781</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="s">
+        <v>507</v>
+      </c>
+      <c r="B22" s="1" t="n">
+        <v>0.340027575486936</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="s">
+        <v>508</v>
+      </c>
+      <c r="B23" s="1" t="n">
+        <v>0.312913062532667</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="1"/>
+    </row>
+    <row r="25">
+      <c r="B25" s="1"/>
+    </row>
+    <row r="26">
+      <c r="B26" s="1"/>
+    </row>
+    <row r="27">
+      <c r="B27" s="1"/>
+    </row>
+    <row r="28">
+      <c r="B28" s="1"/>
+    </row>
+    <row r="29">
+      <c r="B29" s="1"/>
+    </row>
+    <row r="30">
+      <c r="B30" s="1"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100C5B9F2161CEE1040BBC03CB11300495F" ma:contentTypeVersion="12" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="a7cec21613a3259523bdab11a1e26aca">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b5dd4176-d247-4204-85b8-921214f3ccea" xmlns:ns3="359b39ce-e1f9-4933-8424-33b611e6fdcd" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="68943c349d3a016936c8f8cb3335004b" ns2:_="" ns3:_="">
+    <xsd:import namespace="b5dd4176-d247-4204-85b8-921214f3ccea"/>
+    <xsd:import namespace="359b39ce-e1f9-4933-8424-33b611e6fdcd"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="b5dd4176-d247-4204-85b8-921214f3ccea" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="11" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Etiquetas de imagen" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="01529062-7a8b-4d76-943d-e0db5644ee6d" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="15" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="16" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="17" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="18" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="19" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="359b39ce-e1f9-4933-8424-33b611e6fdcd" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="14" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{c9b73259-0823-4f05-8927-4a40ee49fbe1}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="359b39ce-e1f9-4933-8424-33b611e6fdcd">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Tipo de contenido"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Título"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="359b39ce-e1f9-4933-8424-33b611e6fdcd" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b5dd4176-d247-4204-85b8-921214f3ccea">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6258037F-4070-4DD9-8FC2-AC5E529304A1}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{373854D5-8E67-4F7E-B34C-DD3C41A2B84F}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD7BCAAF-C4FA-4526-8313-9941CE068DF5}"/>
 </file>
</xml_diff>

<commit_message>
Corrida | SFE-ID | 2026-03-10 10:15:29.771405
</commit_message>
<xml_diff>
--- a/indicadores/SFE-ID_out.xlsx
+++ b/indicadores/SFE-ID_out.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="509" uniqueCount="509">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="506" uniqueCount="506">
   <si>
     <t xml:space="preserve"/>
   </si>
@@ -1415,19 +1415,10 @@
     <t xml:space="preserve">2030.12</t>
   </si>
   <si>
-    <t xml:space="preserve">Referencias.a.columnas.incluidas.en.la.hoja.DATA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">X2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Columna</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Descripcion</t>
-  </si>
-  <si>
-    <t xml:space="preserve">serie de datos brutos transformados, se importa directo desde base de datos</t>
+    <t xml:space="preserve">REFERENCIA.A.COLUMNAS.INCLUIDAS.EN.LA.HOJA.DATA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">a_original | serie de datos brutos transformados, se importa directo desde base de datos</t>
   </si>
   <si>
     <t xml:space="preserve">a_original_fct_normal | serie original con 12 forecasts obtenidos del mejor modelo ARIMA</t>
@@ -24813,127 +24804,96 @@
       <c r="A1" t="s">
         <v>466</v>
       </c>
-      <c r="B1" t="s">
-        <v>467</v>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>468</v>
-      </c>
-      <c r="B2" t="s">
-        <v>469</v>
+        <v>467</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>34</v>
-      </c>
-      <c r="B3" t="s">
-        <v>470</v>
+        <v>468</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>471</v>
-      </c>
-      <c r="B4"/>
+        <v>469</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>472</v>
-      </c>
-      <c r="B5"/>
+        <v>470</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>473</v>
-      </c>
-      <c r="B6"/>
+        <v>471</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>474</v>
-      </c>
-      <c r="B7"/>
+        <v>472</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>475</v>
-      </c>
-      <c r="B8"/>
+        <v>473</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>476</v>
-      </c>
-      <c r="B9"/>
+        <v>474</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>477</v>
-      </c>
-      <c r="B10"/>
+        <v>475</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>478</v>
-      </c>
-      <c r="B11"/>
+        <v>476</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>479</v>
-      </c>
-      <c r="B12"/>
+        <v>477</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>480</v>
-      </c>
-      <c r="B13"/>
+        <v>478</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>481</v>
-      </c>
-      <c r="B14"/>
+        <v>479</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>482</v>
-      </c>
-      <c r="B15"/>
+        <v>480</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>483</v>
-      </c>
-      <c r="B16"/>
+        <v>481</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>484</v>
-      </c>
-      <c r="B17"/>
+        <v>482</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>485</v>
-      </c>
-      <c r="B18"/>
+        <v>483</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>486</v>
-      </c>
-      <c r="B19"/>
-    </row>
-    <row r="20">
-      <c r="A20" t="s">
-        <v>487</v>
-      </c>
-      <c r="B20"/>
+        <v>484</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -24956,7 +24916,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>488</v>
+        <v>485</v>
       </c>
       <c r="B2" s="1"/>
     </row>
@@ -24966,13 +24926,13 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>489</v>
+        <v>486</v>
       </c>
       <c r="B4" s="1"/>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>490</v>
+        <v>487</v>
       </c>
       <c r="B5" s="1" t="n">
         <v>0.00901068154304649</v>
@@ -24980,7 +24940,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>491</v>
+        <v>488</v>
       </c>
       <c r="B6" s="1" t="n">
         <v>0.0402007093603286</v>
@@ -24988,7 +24948,7 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>492</v>
+        <v>489</v>
       </c>
       <c r="B7" s="1" t="n">
         <v>0.0845682923362035</v>
@@ -24996,7 +24956,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>493</v>
+        <v>490</v>
       </c>
       <c r="B8" s="1" t="n">
         <v>0.161343160115743</v>
@@ -25004,7 +24964,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>494</v>
+        <v>491</v>
       </c>
       <c r="B9" s="1" t="n">
         <v>0.220951473411767</v>
@@ -25012,7 +24972,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>495</v>
+        <v>492</v>
       </c>
       <c r="B10" s="1" t="n">
         <v>0.292950805591597</v>
@@ -25020,7 +24980,7 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>496</v>
+        <v>493</v>
       </c>
       <c r="B11" s="1" t="n">
         <v>0.380874935017229</v>
@@ -25028,7 +24988,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>497</v>
+        <v>494</v>
       </c>
       <c r="B12" s="1" t="n">
         <v>0.451327417048397</v>
@@ -25036,7 +24996,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>498</v>
+        <v>495</v>
       </c>
       <c r="B13" s="1" t="n">
         <v>0.517371477556427</v>
@@ -25044,7 +25004,7 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>499</v>
+        <v>496</v>
       </c>
       <c r="B14" s="1" t="n">
         <v>0.617672515674822</v>
@@ -25052,7 +25012,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>500</v>
+        <v>497</v>
       </c>
       <c r="B15" s="1" t="n">
         <v>0.595737749208721</v>
@@ -25060,7 +25020,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>501</v>
+        <v>498</v>
       </c>
       <c r="B16" s="1" t="n">
         <v>0.578574411724506</v>
@@ -25068,7 +25028,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>502</v>
+        <v>499</v>
       </c>
       <c r="B17" s="1" t="n">
         <v>0.565259695889537</v>
@@ -25076,7 +25036,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>503</v>
+        <v>500</v>
       </c>
       <c r="B18" s="1" t="n">
         <v>0.53004013445323</v>
@@ -25084,7 +25044,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>504</v>
+        <v>501</v>
       </c>
       <c r="B19" s="1" t="n">
         <v>0.535156403669814</v>
@@ -25092,7 +25052,7 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>505</v>
+        <v>502</v>
       </c>
       <c r="B20" s="1" t="n">
         <v>0.475966041991827</v>
@@ -25100,7 +25060,7 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>506</v>
+        <v>503</v>
       </c>
       <c r="B21" s="1" t="n">
         <v>0.388617541773781</v>
@@ -25108,7 +25068,7 @@
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>507</v>
+        <v>504</v>
       </c>
       <c r="B22" s="1" t="n">
         <v>0.340027575486936</v>
@@ -25116,7 +25076,7 @@
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>508</v>
+        <v>505</v>
       </c>
       <c r="B23" s="1" t="n">
         <v>0.312913062532667</v>
@@ -25147,237 +25107,4 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100C5B9F2161CEE1040BBC03CB11300495F" ma:contentTypeVersion="12" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="a7cec21613a3259523bdab11a1e26aca">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b5dd4176-d247-4204-85b8-921214f3ccea" xmlns:ns3="359b39ce-e1f9-4933-8424-33b611e6fdcd" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="68943c349d3a016936c8f8cb3335004b" ns2:_="" ns3:_="">
-    <xsd:import namespace="b5dd4176-d247-4204-85b8-921214f3ccea"/>
-    <xsd:import namespace="359b39ce-e1f9-4933-8424-33b611e6fdcd"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="b5dd4176-d247-4204-85b8-921214f3ccea" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="11" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Etiquetas de imagen" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="01529062-7a8b-4d76-943d-e0db5644ee6d" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="15" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="16" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="17" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="18" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="19" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="359b39ce-e1f9-4933-8424-33b611e6fdcd" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="TaxCatchAll" ma:index="14" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{c9b73259-0823-4f05-8927-4a40ee49fbe1}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="359b39ce-e1f9-4933-8424-33b611e6fdcd">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Tipo de contenido"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Título"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="359b39ce-e1f9-4933-8424-33b611e6fdcd" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b5dd4176-d247-4204-85b8-921214f3ccea">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6258037F-4070-4DD9-8FC2-AC5E529304A1}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{373854D5-8E67-4F7E-B34C-DD3C41A2B84F}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD7BCAAF-C4FA-4526-8313-9941CE068DF5}"/>
 </file>
</xml_diff>

<commit_message>
Corrida | SFE-ID | 2026-03-10 10:18:04.561761
</commit_message>
<xml_diff>
--- a/indicadores/SFE-ID_out.xlsx
+++ b/indicadores/SFE-ID_out.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="506" uniqueCount="506">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="507" uniqueCount="507">
   <si>
     <t xml:space="preserve"/>
   </si>
@@ -1415,7 +1415,10 @@
     <t xml:space="preserve">2030.12</t>
   </si>
   <si>
-    <t xml:space="preserve">REFERENCIA.A.COLUMNAS.INCLUIDAS.EN.LA.HOJA.DATA</t>
+    <t xml:space="preserve">FRANCO.OCAMPO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REFERENCIA A COLUMNAS INCLUIDAS EN LA HOJA DATA</t>
   </si>
   <si>
     <t xml:space="preserve">a_original | serie de datos brutos transformados, se importa directo desde base de datos</t>
@@ -24895,6 +24898,11 @@
         <v>484</v>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" t="s">
+        <v>485</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
@@ -24916,7 +24924,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="B2" s="1"/>
     </row>
@@ -24926,13 +24934,13 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="B4" s="1"/>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="B5" s="1" t="n">
         <v>0.00901068154304649</v>
@@ -24940,7 +24948,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="B6" s="1" t="n">
         <v>0.0402007093603286</v>
@@ -24948,7 +24956,7 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="B7" s="1" t="n">
         <v>0.0845682923362035</v>
@@ -24956,7 +24964,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="B8" s="1" t="n">
         <v>0.161343160115743</v>
@@ -24964,7 +24972,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="B9" s="1" t="n">
         <v>0.220951473411767</v>
@@ -24972,7 +24980,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="B10" s="1" t="n">
         <v>0.292950805591597</v>
@@ -24980,7 +24988,7 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="B11" s="1" t="n">
         <v>0.380874935017229</v>
@@ -24988,7 +24996,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="B12" s="1" t="n">
         <v>0.451327417048397</v>
@@ -24996,7 +25004,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="B13" s="1" t="n">
         <v>0.517371477556427</v>
@@ -25004,7 +25012,7 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="B14" s="1" t="n">
         <v>0.617672515674822</v>
@@ -25012,7 +25020,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="B15" s="1" t="n">
         <v>0.595737749208721</v>
@@ -25020,7 +25028,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="B16" s="1" t="n">
         <v>0.578574411724506</v>
@@ -25028,7 +25036,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="B17" s="1" t="n">
         <v>0.565259695889537</v>
@@ -25036,7 +25044,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="B18" s="1" t="n">
         <v>0.53004013445323</v>
@@ -25044,7 +25052,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="B19" s="1" t="n">
         <v>0.535156403669814</v>
@@ -25052,7 +25060,7 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="B20" s="1" t="n">
         <v>0.475966041991827</v>
@@ -25060,7 +25068,7 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="B21" s="1" t="n">
         <v>0.388617541773781</v>
@@ -25068,7 +25076,7 @@
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="B22" s="1" t="n">
         <v>0.340027575486936</v>
@@ -25076,7 +25084,7 @@
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="B23" s="1" t="n">
         <v>0.312913062532667</v>

</xml_diff>

<commit_message>
Corrida | SFE-ID | 2026-03-10 11:21:40.617283
</commit_message>
<xml_diff>
--- a/indicadores/SFE-ID_out.xlsx
+++ b/indicadores/SFE-ID_out.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="507" uniqueCount="507">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="506" uniqueCount="506">
   <si>
     <t xml:space="preserve"/>
   </si>
@@ -1415,10 +1415,7 @@
     <t xml:space="preserve">2030.12</t>
   </si>
   <si>
-    <t xml:space="preserve">X1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">REFERENCIA A COLUMNAS INCLUIDAS EN LA HOJA DATA</t>
+    <t xml:space="preserve">Referencias de las series incluidas en la hoja Data</t>
   </si>
   <si>
     <t xml:space="preserve">a_original | serie de datos brutos transformados, se importa directo desde base de datos</t>
@@ -24898,11 +24895,6 @@
         <v>484</v>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" t="s">
-        <v>485</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
@@ -24924,7 +24916,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="B2" s="1"/>
     </row>
@@ -24934,13 +24926,13 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="B4" s="1"/>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="B5" s="1" t="n">
         <v>0.00901068154304649</v>
@@ -24948,7 +24940,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="B6" s="1" t="n">
         <v>0.0402007093603286</v>
@@ -24956,7 +24948,7 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="B7" s="1" t="n">
         <v>0.0845682923362035</v>
@@ -24964,7 +24956,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="B8" s="1" t="n">
         <v>0.161343160115743</v>
@@ -24972,7 +24964,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="B9" s="1" t="n">
         <v>0.220951473411767</v>
@@ -24980,7 +24972,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="B10" s="1" t="n">
         <v>0.292950805591597</v>
@@ -24988,7 +24980,7 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="B11" s="1" t="n">
         <v>0.380874935017229</v>
@@ -24996,7 +24988,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="B12" s="1" t="n">
         <v>0.451327417048397</v>
@@ -25004,7 +24996,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="B13" s="1" t="n">
         <v>0.517371477556427</v>
@@ -25012,7 +25004,7 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="B14" s="1" t="n">
         <v>0.617672515674822</v>
@@ -25020,7 +25012,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
       <c r="B15" s="1" t="n">
         <v>0.595737749208721</v>
@@ -25028,7 +25020,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="B16" s="1" t="n">
         <v>0.578574411724506</v>
@@ -25036,7 +25028,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="B17" s="1" t="n">
         <v>0.565259695889537</v>
@@ -25044,7 +25036,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="B18" s="1" t="n">
         <v>0.53004013445323</v>
@@ -25052,7 +25044,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="B19" s="1" t="n">
         <v>0.535156403669814</v>
@@ -25060,7 +25052,7 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="B20" s="1" t="n">
         <v>0.475966041991827</v>
@@ -25068,7 +25060,7 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="B21" s="1" t="n">
         <v>0.388617541773781</v>
@@ -25076,7 +25068,7 @@
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="B22" s="1" t="n">
         <v>0.340027575486936</v>
@@ -25084,7 +25076,7 @@
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="B23" s="1" t="n">
         <v>0.312913062532667</v>

</xml_diff>

<commit_message>
Corrida | SFE-ID | 2026-03-17 08:59:45.901321
</commit_message>
<xml_diff>
--- a/indicadores/SFE-ID_out.xlsx
+++ b/indicadores/SFE-ID_out.xlsx
@@ -107,13 +107,13 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">10/03/2026</t>
+    <t xml:space="preserve">17/03/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
   </si>
   <si>
-    <t xml:space="preserve">focampo</t>
+    <t xml:space="preserve">pcohan</t>
   </si>
   <si>
     <t xml:space="preserve">fecha</t>
@@ -2066,7 +2066,7 @@
       <c r="B9"/>
       <c r="C9"/>
       <c r="D9" t="n">
-        <v>0.617672515674822</v>
+        <v>0.618246701165947</v>
       </c>
       <c r="E9"/>
       <c r="F9"/>
@@ -2124,7 +2124,7 @@
       <c r="B13"/>
       <c r="C13"/>
       <c r="D13" t="n">
-        <v>0.381519336620063</v>
+        <v>0.382228983502577</v>
       </c>
       <c r="E13"/>
       <c r="F13"/>
@@ -2194,7 +2194,7 @@
       <c r="B18"/>
       <c r="C18"/>
       <c r="D18" t="n">
-        <v>0.778576546768402</v>
+        <v>0.786009399979254</v>
       </c>
       <c r="E18"/>
       <c r="F18"/>
@@ -2224,7 +2224,7 @@
       <c r="B20"/>
       <c r="C20"/>
       <c r="D20" t="n">
-        <v>0.0000000901456629530707</v>
+        <v>0.0000000877804493973573</v>
       </c>
       <c r="E20"/>
       <c r="F20"/>
@@ -24935,7 +24935,7 @@
         <v>487</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>0.00901068154304649</v>
+        <v>0.00850051953671227</v>
       </c>
     </row>
     <row r="6">
@@ -24943,7 +24943,7 @@
         <v>488</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>0.0402007093603286</v>
+        <v>0.0401968358117712</v>
       </c>
     </row>
     <row r="7">
@@ -24951,7 +24951,7 @@
         <v>489</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>0.0845682923362035</v>
+        <v>0.0858524656448025</v>
       </c>
     </row>
     <row r="8">
@@ -24959,7 +24959,7 @@
         <v>490</v>
       </c>
       <c r="B8" s="1" t="n">
-        <v>0.161343160115743</v>
+        <v>0.162960989941894</v>
       </c>
     </row>
     <row r="9">
@@ -24967,7 +24967,7 @@
         <v>491</v>
       </c>
       <c r="B9" s="1" t="n">
-        <v>0.220951473411767</v>
+        <v>0.223172083532713</v>
       </c>
     </row>
     <row r="10">
@@ -24975,7 +24975,7 @@
         <v>492</v>
       </c>
       <c r="B10" s="1" t="n">
-        <v>0.292950805591597</v>
+        <v>0.294727309351349</v>
       </c>
     </row>
     <row r="11">
@@ -24983,7 +24983,7 @@
         <v>493</v>
       </c>
       <c r="B11" s="1" t="n">
-        <v>0.380874935017229</v>
+        <v>0.382059320975483</v>
       </c>
     </row>
     <row r="12">
@@ -24991,7 +24991,7 @@
         <v>494</v>
       </c>
       <c r="B12" s="1" t="n">
-        <v>0.451327417048397</v>
+        <v>0.452727514903291</v>
       </c>
     </row>
     <row r="13">
@@ -24999,7 +24999,7 @@
         <v>495</v>
       </c>
       <c r="B13" s="1" t="n">
-        <v>0.517371477556427</v>
+        <v>0.518775572086454</v>
       </c>
     </row>
     <row r="14">
@@ -25007,7 +25007,7 @@
         <v>496</v>
       </c>
       <c r="B14" s="1" t="n">
-        <v>0.617672515674822</v>
+        <v>0.618246701165947</v>
       </c>
     </row>
     <row r="15">
@@ -25015,7 +25015,7 @@
         <v>497</v>
       </c>
       <c r="B15" s="1" t="n">
-        <v>0.595737749208721</v>
+        <v>0.595242606728072</v>
       </c>
     </row>
     <row r="16">
@@ -25023,7 +25023,7 @@
         <v>498</v>
       </c>
       <c r="B16" s="1" t="n">
-        <v>0.578574411724506</v>
+        <v>0.578829838174496</v>
       </c>
     </row>
     <row r="17">
@@ -25031,7 +25031,7 @@
         <v>499</v>
       </c>
       <c r="B17" s="1" t="n">
-        <v>0.565259695889537</v>
+        <v>0.564024753152211</v>
       </c>
     </row>
     <row r="18">
@@ -25039,7 +25039,7 @@
         <v>500</v>
       </c>
       <c r="B18" s="1" t="n">
-        <v>0.53004013445323</v>
+        <v>0.529098125877195</v>
       </c>
     </row>
     <row r="19">
@@ -25047,7 +25047,7 @@
         <v>501</v>
       </c>
       <c r="B19" s="1" t="n">
-        <v>0.535156403669814</v>
+        <v>0.534048474240756</v>
       </c>
     </row>
     <row r="20">
@@ -25055,7 +25055,7 @@
         <v>502</v>
       </c>
       <c r="B20" s="1" t="n">
-        <v>0.475966041991827</v>
+        <v>0.474390075227322</v>
       </c>
     </row>
     <row r="21">
@@ -25063,7 +25063,7 @@
         <v>503</v>
       </c>
       <c r="B21" s="1" t="n">
-        <v>0.388617541773781</v>
+        <v>0.386868747276603</v>
       </c>
     </row>
     <row r="22">
@@ -25071,7 +25071,7 @@
         <v>504</v>
       </c>
       <c r="B22" s="1" t="n">
-        <v>0.340027575486936</v>
+        <v>0.33791497645484</v>
       </c>
     </row>
     <row r="23">
@@ -25079,7 +25079,7 @@
         <v>505</v>
       </c>
       <c r="B23" s="1" t="n">
-        <v>0.312913062532667</v>
+        <v>0.311254989601045</v>
       </c>
     </row>
     <row r="24">

</xml_diff>

<commit_message>
Corrida | SFE-ID | 2026-05-07 08:52:09.86099
</commit_message>
<xml_diff>
--- a/indicadores/SFE-ID_out.xlsx
+++ b/indicadores/SFE-ID_out.xlsx
@@ -107,13 +107,13 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">16/04/2026</t>
+    <t xml:space="preserve">07/05/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
   </si>
   <si>
-    <t xml:space="preserve">pcohan</t>
+    <t xml:space="preserve">franco</t>
   </si>
   <si>
     <t xml:space="preserve">fecha</t>
@@ -2066,7 +2066,7 @@
       <c r="B9"/>
       <c r="C9"/>
       <c r="D9" t="n">
-        <v>0.617799912695538</v>
+        <v>0.618377169932261</v>
       </c>
       <c r="E9"/>
       <c r="F9"/>
@@ -2124,7 +2124,7 @@
       <c r="B13"/>
       <c r="C13"/>
       <c r="D13" t="n">
-        <v>0.381676732126615</v>
+        <v>0.382390324293432</v>
       </c>
       <c r="E13"/>
       <c r="F13"/>
@@ -2194,7 +2194,7 @@
       <c r="B18"/>
       <c r="C18"/>
       <c r="D18" t="n">
-        <v>0.777326317722256</v>
+        <v>0.734164515054875</v>
       </c>
       <c r="E18"/>
       <c r="F18"/>
@@ -2224,7 +2224,7 @@
       <c r="B20"/>
       <c r="C20"/>
       <c r="D20" t="n">
-        <v>0.0000000582038672380905</v>
+        <v>0.0000000738565564010493</v>
       </c>
       <c r="E20"/>
       <c r="F20"/>
@@ -25007,7 +25007,7 @@
         <v>487</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>0.00883687919996099</v>
+        <v>0.00595348433252861</v>
       </c>
     </row>
     <row r="6">
@@ -25015,7 +25015,7 @@
         <v>488</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>0.0397453853163336</v>
+        <v>0.0370376963655155</v>
       </c>
     </row>
     <row r="7">
@@ -25023,7 +25023,7 @@
         <v>489</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>0.087076523485903</v>
+        <v>0.083431584912265</v>
       </c>
     </row>
     <row r="8">
@@ -25031,7 +25031,7 @@
         <v>490</v>
       </c>
       <c r="B8" s="1" t="n">
-        <v>0.162452227208012</v>
+        <v>0.16132502728309</v>
       </c>
     </row>
     <row r="9">
@@ -25039,7 +25039,7 @@
         <v>491</v>
       </c>
       <c r="B9" s="1" t="n">
-        <v>0.2229218366962</v>
+        <v>0.220855896533849</v>
       </c>
     </row>
     <row r="10">
@@ -25047,7 +25047,7 @@
         <v>492</v>
       </c>
       <c r="B10" s="1" t="n">
-        <v>0.295365741770121</v>
+        <v>0.293470262425822</v>
       </c>
     </row>
     <row r="11">
@@ -25055,7 +25055,7 @@
         <v>493</v>
       </c>
       <c r="B11" s="1" t="n">
-        <v>0.381837872094801</v>
+        <v>0.381995723974717</v>
       </c>
     </row>
     <row r="12">
@@ -25063,7 +25063,7 @@
         <v>494</v>
       </c>
       <c r="B12" s="1" t="n">
-        <v>0.452609625845966</v>
+        <v>0.452220451300217</v>
       </c>
     </row>
     <row r="13">
@@ -25071,7 +25071,7 @@
         <v>495</v>
       </c>
       <c r="B13" s="1" t="n">
-        <v>0.517889060331753</v>
+        <v>0.5179227588009</v>
       </c>
     </row>
     <row r="14">
@@ -25079,7 +25079,7 @@
         <v>496</v>
       </c>
       <c r="B14" s="1" t="n">
-        <v>0.617799912695538</v>
+        <v>0.618377169932261</v>
       </c>
     </row>
     <row r="15">
@@ -25087,7 +25087,7 @@
         <v>497</v>
       </c>
       <c r="B15" s="1" t="n">
-        <v>0.594059392693297</v>
+        <v>0.59409277274735</v>
       </c>
     </row>
     <row r="16">
@@ -25095,7 +25095,7 @@
         <v>498</v>
       </c>
       <c r="B16" s="1" t="n">
-        <v>0.578033277249742</v>
+        <v>0.577073896257431</v>
       </c>
     </row>
     <row r="17">
@@ -25103,7 +25103,7 @@
         <v>499</v>
       </c>
       <c r="B17" s="1" t="n">
-        <v>0.564081390531816</v>
+        <v>0.562455061781831</v>
       </c>
     </row>
     <row r="18">
@@ -25111,7 +25111,7 @@
         <v>500</v>
       </c>
       <c r="B18" s="1" t="n">
-        <v>0.530342353375101</v>
+        <v>0.529677480727779</v>
       </c>
     </row>
     <row r="19">
@@ -25119,7 +25119,7 @@
         <v>501</v>
       </c>
       <c r="B19" s="1" t="n">
-        <v>0.537081714015482</v>
+        <v>0.536767212562935</v>
       </c>
     </row>
     <row r="20">
@@ -25127,7 +25127,7 @@
         <v>502</v>
       </c>
       <c r="B20" s="1" t="n">
-        <v>0.476872813122936</v>
+        <v>0.477265699357675</v>
       </c>
     </row>
     <row r="21">
@@ -25135,7 +25135,7 @@
         <v>503</v>
       </c>
       <c r="B21" s="1" t="n">
-        <v>0.386153821191053</v>
+        <v>0.387720101004318</v>
       </c>
     </row>
     <row r="22">
@@ -25143,7 +25143,7 @@
         <v>504</v>
       </c>
       <c r="B22" s="1" t="n">
-        <v>0.337200697257554</v>
+        <v>0.338123324824612</v>
       </c>
     </row>
     <row r="23">
@@ -25151,7 +25151,7 @@
         <v>505</v>
       </c>
       <c r="B23" s="1" t="n">
-        <v>0.310578018366052</v>
+        <v>0.310838097706036</v>
       </c>
     </row>
     <row r="24">
@@ -25179,4 +25179,237 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100C5B9F2161CEE1040BBC03CB11300495F" ma:contentTypeVersion="12" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="4b8b282811f2bcc11ff842570f663f4a">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b5dd4176-d247-4204-85b8-921214f3ccea" xmlns:ns3="359b39ce-e1f9-4933-8424-33b611e6fdcd" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="8b7f2ae8e4517a268e1f460c8f9cedce" ns2:_="" ns3:_="">
+    <xsd:import namespace="b5dd4176-d247-4204-85b8-921214f3ccea"/>
+    <xsd:import namespace="359b39ce-e1f9-4933-8424-33b611e6fdcd"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="b5dd4176-d247-4204-85b8-921214f3ccea" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="11" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="01529062-7a8b-4d76-943d-e0db5644ee6d" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="15" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="16" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="17" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="18" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="19" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="359b39ce-e1f9-4933-8424-33b611e6fdcd" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="14" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{c9b73259-0823-4f05-8927-4a40ee49fbe1}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="359b39ce-e1f9-4933-8424-33b611e6fdcd">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b5dd4176-d247-4204-85b8-921214f3ccea">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="359b39ce-e1f9-4933-8424-33b611e6fdcd" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{61C81EEF-0D9A-40B9-B94A-6018010BD86A}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7197C1AC-BF24-41CE-87F7-2A08110A932C}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5FEA8798-8FE0-4BE3-9239-A5FA65FE6455}"/>
 </file>
</xml_diff>

<commit_message>
Corrida | SFE-ID | 2026-05-08 11:56:20.442861
</commit_message>
<xml_diff>
--- a/indicadores/SFE-ID_out.xlsx
+++ b/indicadores/SFE-ID_out.xlsx
@@ -107,13 +107,13 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">07/05/2026</t>
+    <t xml:space="preserve">08/05/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
   </si>
   <si>
-    <t xml:space="preserve">franco</t>
+    <t xml:space="preserve">pcohan</t>
   </si>
   <si>
     <t xml:space="preserve">fecha</t>
@@ -25179,237 +25179,4 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100C5B9F2161CEE1040BBC03CB11300495F" ma:contentTypeVersion="12" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="4b8b282811f2bcc11ff842570f663f4a">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b5dd4176-d247-4204-85b8-921214f3ccea" xmlns:ns3="359b39ce-e1f9-4933-8424-33b611e6fdcd" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="8b7f2ae8e4517a268e1f460c8f9cedce" ns2:_="" ns3:_="">
-    <xsd:import namespace="b5dd4176-d247-4204-85b8-921214f3ccea"/>
-    <xsd:import namespace="359b39ce-e1f9-4933-8424-33b611e6fdcd"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="b5dd4176-d247-4204-85b8-921214f3ccea" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="11" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="01529062-7a8b-4d76-943d-e0db5644ee6d" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="15" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="16" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="17" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="18" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="19" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="359b39ce-e1f9-4933-8424-33b611e6fdcd" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="TaxCatchAll" ma:index="14" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{c9b73259-0823-4f05-8927-4a40ee49fbe1}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="359b39ce-e1f9-4933-8424-33b611e6fdcd">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b5dd4176-d247-4204-85b8-921214f3ccea">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="359b39ce-e1f9-4933-8424-33b611e6fdcd" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{61C81EEF-0D9A-40B9-B94A-6018010BD86A}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7197C1AC-BF24-41CE-87F7-2A08110A932C}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5FEA8798-8FE0-4BE3-9239-A5FA65FE6455}"/>
 </file>
</xml_diff>

<commit_message>
Corrida | SFE-ID | 2026-05-12 09:26:43.758158
</commit_message>
<xml_diff>
--- a/indicadores/SFE-ID_out.xlsx
+++ b/indicadores/SFE-ID_out.xlsx
@@ -107,13 +107,13 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">08/05/2026</t>
+    <t xml:space="preserve">12/05/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
   </si>
   <si>
-    <t xml:space="preserve">pcohan</t>
+    <t xml:space="preserve">focampo</t>
   </si>
   <si>
     <t xml:space="preserve">fecha</t>

</xml_diff>

<commit_message>
Corrida | SFE-ID | 2026-05-18 08:47:01.77612
</commit_message>
<xml_diff>
--- a/indicadores/SFE-ID_out.xlsx
+++ b/indicadores/SFE-ID_out.xlsx
@@ -107,13 +107,13 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">15/05/2026</t>
+    <t xml:space="preserve">18/05/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
   </si>
   <si>
-    <t xml:space="preserve">arodriguez</t>
+    <t xml:space="preserve">focampo</t>
   </si>
   <si>
     <t xml:space="preserve">fecha</t>
@@ -2066,7 +2066,7 @@
       <c r="B9"/>
       <c r="C9"/>
       <c r="D9" t="n">
-        <v>0.617722874264605</v>
+        <v>0.625566835747602</v>
       </c>
       <c r="E9"/>
       <c r="F9"/>
@@ -2124,7 +2124,7 @@
       <c r="B13"/>
       <c r="C13"/>
       <c r="D13" t="n">
-        <v>0.381581549389725</v>
+        <v>0.391333865987267</v>
       </c>
       <c r="E13"/>
       <c r="F13"/>
@@ -2194,7 +2194,7 @@
       <c r="B18"/>
       <c r="C18"/>
       <c r="D18" t="n">
-        <v>0.73073464748252</v>
+        <v>0.860218954818676</v>
       </c>
       <c r="E18"/>
       <c r="F18"/>
@@ -2224,7 +2224,7 @@
       <c r="B20"/>
       <c r="C20"/>
       <c r="D20" t="n">
-        <v>0.0000000648754502203118</v>
+        <v>0.0000000458850409216531</v>
       </c>
       <c r="E20"/>
       <c r="F20"/>
@@ -25043,7 +25043,7 @@
         <v>487</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>0.00534672665980023</v>
+        <v>0.00627218327481068</v>
       </c>
     </row>
     <row r="6">
@@ -25051,7 +25051,7 @@
         <v>488</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>0.0368626814363363</v>
+        <v>0.0372689757434773</v>
       </c>
     </row>
     <row r="7">
@@ -25059,7 +25059,7 @@
         <v>489</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>0.0834718206458405</v>
+        <v>0.0867115899421955</v>
       </c>
     </row>
     <row r="8">
@@ -25067,7 +25067,7 @@
         <v>490</v>
       </c>
       <c r="B8" s="1" t="n">
-        <v>0.161553871487426</v>
+        <v>0.165107765005101</v>
       </c>
     </row>
     <row r="9">
@@ -25075,7 +25075,7 @@
         <v>491</v>
       </c>
       <c r="B9" s="1" t="n">
-        <v>0.221009097229986</v>
+        <v>0.227203373507679</v>
       </c>
     </row>
     <row r="10">
@@ -25083,7 +25083,7 @@
         <v>492</v>
       </c>
       <c r="B10" s="1" t="n">
-        <v>0.293335206054956</v>
+        <v>0.299268046831524</v>
       </c>
     </row>
     <row r="11">
@@ -25091,7 +25091,7 @@
         <v>493</v>
       </c>
       <c r="B11" s="1" t="n">
-        <v>0.381653865760621</v>
+        <v>0.378705420798249</v>
       </c>
     </row>
     <row r="12">
@@ -25099,7 +25099,7 @@
         <v>494</v>
       </c>
       <c r="B12" s="1" t="n">
-        <v>0.451711434626133</v>
+        <v>0.44947616653041</v>
       </c>
     </row>
     <row r="13">
@@ -25107,7 +25107,7 @@
         <v>495</v>
       </c>
       <c r="B13" s="1" t="n">
-        <v>0.517255513664941</v>
+        <v>0.522418729362734</v>
       </c>
     </row>
     <row r="14">
@@ -25115,7 +25115,7 @@
         <v>496</v>
       </c>
       <c r="B14" s="1" t="n">
-        <v>0.617722874264605</v>
+        <v>0.625566835747602</v>
       </c>
     </row>
     <row r="15">
@@ -25123,7 +25123,7 @@
         <v>497</v>
       </c>
       <c r="B15" s="1" t="n">
-        <v>0.593251907452273</v>
+        <v>0.599102127819066</v>
       </c>
     </row>
     <row r="16">
@@ -25131,7 +25131,7 @@
         <v>498</v>
       </c>
       <c r="B16" s="1" t="n">
-        <v>0.576591603839801</v>
+        <v>0.578416398489107</v>
       </c>
     </row>
     <row r="17">
@@ -25139,7 +25139,7 @@
         <v>499</v>
       </c>
       <c r="B17" s="1" t="n">
-        <v>0.562537415694473</v>
+        <v>0.562233295475917</v>
       </c>
     </row>
     <row r="18">
@@ -25147,7 +25147,7 @@
         <v>500</v>
       </c>
       <c r="B18" s="1" t="n">
-        <v>0.529276060772297</v>
+        <v>0.526639462347366</v>
       </c>
     </row>
     <row r="19">
@@ -25155,7 +25155,7 @@
         <v>501</v>
       </c>
       <c r="B19" s="1" t="n">
-        <v>0.536405305398364</v>
+        <v>0.531190921089674</v>
       </c>
     </row>
     <row r="20">
@@ -25163,7 +25163,7 @@
         <v>502</v>
       </c>
       <c r="B20" s="1" t="n">
-        <v>0.477097667669728</v>
+        <v>0.473452983724756</v>
       </c>
     </row>
     <row r="21">
@@ -25171,7 +25171,7 @@
         <v>503</v>
       </c>
       <c r="B21" s="1" t="n">
-        <v>0.387896704460275</v>
+        <v>0.384708445735832</v>
       </c>
     </row>
     <row r="22">
@@ -25179,7 +25179,7 @@
         <v>504</v>
       </c>
       <c r="B22" s="1" t="n">
-        <v>0.33945668294405</v>
+        <v>0.339754649660267</v>
       </c>
     </row>
     <row r="23">
@@ -25187,7 +25187,7 @@
         <v>505</v>
       </c>
       <c r="B23" s="1" t="n">
-        <v>0.31224617454051</v>
+        <v>0.319206321457706</v>
       </c>
     </row>
     <row r="24">

</xml_diff>

<commit_message>
Corrida | SFE-ID | 2026-05-19 14:00:09.656238
</commit_message>
<xml_diff>
--- a/indicadores/SFE-ID_out.xlsx
+++ b/indicadores/SFE-ID_out.xlsx
@@ -107,7 +107,7 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">18/05/2026</t>
+    <t xml:space="preserve">19/05/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
@@ -2066,7 +2066,7 @@
       <c r="B9"/>
       <c r="C9"/>
       <c r="D9" t="n">
-        <v>0.625566835747602</v>
+        <v>0.625546250468052</v>
       </c>
       <c r="E9"/>
       <c r="F9"/>
@@ -2124,7 +2124,7 @@
       <c r="B13"/>
       <c r="C13"/>
       <c r="D13" t="n">
-        <v>0.391333865987267</v>
+        <v>0.391308111474639</v>
       </c>
       <c r="E13"/>
       <c r="F13"/>
@@ -2194,7 +2194,7 @@
       <c r="B18"/>
       <c r="C18"/>
       <c r="D18" t="n">
-        <v>0.860218954818676</v>
+        <v>0.856555515249729</v>
       </c>
       <c r="E18"/>
       <c r="F18"/>
@@ -2224,7 +2224,7 @@
       <c r="B20"/>
       <c r="C20"/>
       <c r="D20" t="n">
-        <v>0.0000000458850409216531</v>
+        <v>0.0000000487860572060122</v>
       </c>
       <c r="E20"/>
       <c r="F20"/>
@@ -25043,7 +25043,7 @@
         <v>487</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>0.00627218327481068</v>
+        <v>0.00607234423208874</v>
       </c>
     </row>
     <row r="6">
@@ -25051,7 +25051,7 @@
         <v>488</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>0.0372689757434773</v>
+        <v>0.0370795636598727</v>
       </c>
     </row>
     <row r="7">
@@ -25059,7 +25059,7 @@
         <v>489</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>0.0867115899421955</v>
+        <v>0.0862335743062676</v>
       </c>
     </row>
     <row r="8">
@@ -25067,7 +25067,7 @@
         <v>490</v>
       </c>
       <c r="B8" s="1" t="n">
-        <v>0.165107765005101</v>
+        <v>0.16571416732658</v>
       </c>
     </row>
     <row r="9">
@@ -25075,7 +25075,7 @@
         <v>491</v>
       </c>
       <c r="B9" s="1" t="n">
-        <v>0.227203373507679</v>
+        <v>0.226865673480195</v>
       </c>
     </row>
     <row r="10">
@@ -25083,7 +25083,7 @@
         <v>492</v>
       </c>
       <c r="B10" s="1" t="n">
-        <v>0.299268046831524</v>
+        <v>0.299230027663466</v>
       </c>
     </row>
     <row r="11">
@@ -25091,7 +25091,7 @@
         <v>493</v>
       </c>
       <c r="B11" s="1" t="n">
-        <v>0.378705420798249</v>
+        <v>0.378354413743636</v>
       </c>
     </row>
     <row r="12">
@@ -25099,7 +25099,7 @@
         <v>494</v>
       </c>
       <c r="B12" s="1" t="n">
-        <v>0.44947616653041</v>
+        <v>0.449292416452931</v>
       </c>
     </row>
     <row r="13">
@@ -25107,7 +25107,7 @@
         <v>495</v>
       </c>
       <c r="B13" s="1" t="n">
-        <v>0.522418729362734</v>
+        <v>0.522140195792422</v>
       </c>
     </row>
     <row r="14">
@@ -25115,7 +25115,7 @@
         <v>496</v>
       </c>
       <c r="B14" s="1" t="n">
-        <v>0.625566835747602</v>
+        <v>0.625546250468052</v>
       </c>
     </row>
     <row r="15">
@@ -25123,7 +25123,7 @@
         <v>497</v>
       </c>
       <c r="B15" s="1" t="n">
-        <v>0.599102127819066</v>
+        <v>0.598619182763922</v>
       </c>
     </row>
     <row r="16">
@@ -25131,7 +25131,7 @@
         <v>498</v>
       </c>
       <c r="B16" s="1" t="n">
-        <v>0.578416398489107</v>
+        <v>0.578064618043328</v>
       </c>
     </row>
     <row r="17">
@@ -25139,7 +25139,7 @@
         <v>499</v>
       </c>
       <c r="B17" s="1" t="n">
-        <v>0.562233295475917</v>
+        <v>0.561614954578717</v>
       </c>
     </row>
     <row r="18">
@@ -25147,7 +25147,7 @@
         <v>500</v>
       </c>
       <c r="B18" s="1" t="n">
-        <v>0.526639462347366</v>
+        <v>0.525786860392088</v>
       </c>
     </row>
     <row r="19">
@@ -25155,7 +25155,7 @@
         <v>501</v>
       </c>
       <c r="B19" s="1" t="n">
-        <v>0.531190921089674</v>
+        <v>0.530313709735418</v>
       </c>
     </row>
     <row r="20">
@@ -25163,7 +25163,7 @@
         <v>502</v>
       </c>
       <c r="B20" s="1" t="n">
-        <v>0.473452983724756</v>
+        <v>0.472540300670596</v>
       </c>
     </row>
     <row r="21">
@@ -25171,7 +25171,7 @@
         <v>503</v>
       </c>
       <c r="B21" s="1" t="n">
-        <v>0.384708445735832</v>
+        <v>0.384287779944996</v>
       </c>
     </row>
     <row r="22">
@@ -25179,7 +25179,7 @@
         <v>504</v>
       </c>
       <c r="B22" s="1" t="n">
-        <v>0.339754649660267</v>
+        <v>0.340115405485498</v>
       </c>
     </row>
     <row r="23">
@@ -25187,7 +25187,7 @@
         <v>505</v>
       </c>
       <c r="B23" s="1" t="n">
-        <v>0.319206321457706</v>
+        <v>0.31988896805625</v>
       </c>
     </row>
     <row r="24">

</xml_diff>

<commit_message>
Corrida | SFE-ID | 2026-06-01 12:11:48.852134
</commit_message>
<xml_diff>
--- a/indicadores/SFE-ID_out.xlsx
+++ b/indicadores/SFE-ID_out.xlsx
@@ -107,13 +107,13 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">19/05/2026</t>
+    <t xml:space="preserve">01/06/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
   </si>
   <si>
-    <t xml:space="preserve">pcohan</t>
+    <t xml:space="preserve">focampo</t>
   </si>
   <si>
     <t xml:space="preserve">fecha</t>
@@ -2066,7 +2066,7 @@
       <c r="B9"/>
       <c r="C9"/>
       <c r="D9" t="n">
-        <v>0.625546250468052</v>
+        <v>0.624569729143181</v>
       </c>
       <c r="E9"/>
       <c r="F9"/>
@@ -2124,7 +2124,7 @@
       <c r="B13"/>
       <c r="C13"/>
       <c r="D13" t="n">
-        <v>0.391308111474639</v>
+        <v>0.390087346561987</v>
       </c>
       <c r="E13"/>
       <c r="F13"/>
@@ -2194,7 +2194,7 @@
       <c r="B18"/>
       <c r="C18"/>
       <c r="D18" t="n">
-        <v>0.856555515249729</v>
+        <v>0.839680606890857</v>
       </c>
       <c r="E18"/>
       <c r="F18"/>
@@ -2224,7 +2224,7 @@
       <c r="B20"/>
       <c r="C20"/>
       <c r="D20" t="n">
-        <v>0.0000000487860572060122</v>
+        <v>0.0000000555893859833005</v>
       </c>
       <c r="E20"/>
       <c r="F20"/>
@@ -25043,7 +25043,7 @@
         <v>487</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>0.00607234423208874</v>
+        <v>0.00500732690276153</v>
       </c>
     </row>
     <row r="6">
@@ -25051,7 +25051,7 @@
         <v>488</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>0.0370795636598727</v>
+        <v>0.0355257410207497</v>
       </c>
     </row>
     <row r="7">
@@ -25059,7 +25059,7 @@
         <v>489</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>0.0862335743062676</v>
+        <v>0.0846452366350987</v>
       </c>
     </row>
     <row r="8">
@@ -25067,7 +25067,7 @@
         <v>490</v>
       </c>
       <c r="B8" s="1" t="n">
-        <v>0.16571416732658</v>
+        <v>0.16551753995147</v>
       </c>
     </row>
     <row r="9">
@@ -25075,7 +25075,7 @@
         <v>491</v>
       </c>
       <c r="B9" s="1" t="n">
-        <v>0.226865673480195</v>
+        <v>0.226973551786283</v>
       </c>
     </row>
     <row r="10">
@@ -25083,7 +25083,7 @@
         <v>492</v>
       </c>
       <c r="B10" s="1" t="n">
-        <v>0.299230027663466</v>
+        <v>0.299660335941655</v>
       </c>
     </row>
     <row r="11">
@@ -25091,7 +25091,7 @@
         <v>493</v>
       </c>
       <c r="B11" s="1" t="n">
-        <v>0.378354413743636</v>
+        <v>0.378603183111057</v>
       </c>
     </row>
     <row r="12">
@@ -25099,7 +25099,7 @@
         <v>494</v>
       </c>
       <c r="B12" s="1" t="n">
-        <v>0.449292416452931</v>
+        <v>0.449949381821148</v>
       </c>
     </row>
     <row r="13">
@@ -25107,7 +25107,7 @@
         <v>495</v>
       </c>
       <c r="B13" s="1" t="n">
-        <v>0.522140195792422</v>
+        <v>0.522446243289262</v>
       </c>
     </row>
     <row r="14">
@@ -25115,7 +25115,7 @@
         <v>496</v>
       </c>
       <c r="B14" s="1" t="n">
-        <v>0.625546250468052</v>
+        <v>0.624569729143181</v>
       </c>
     </row>
     <row r="15">
@@ -25123,7 +25123,7 @@
         <v>497</v>
       </c>
       <c r="B15" s="1" t="n">
-        <v>0.598619182763922</v>
+        <v>0.598132854598252</v>
       </c>
     </row>
     <row r="16">
@@ -25131,7 +25131,7 @@
         <v>498</v>
       </c>
       <c r="B16" s="1" t="n">
-        <v>0.578064618043328</v>
+        <v>0.57823903340475</v>
       </c>
     </row>
     <row r="17">
@@ -25139,7 +25139,7 @@
         <v>499</v>
       </c>
       <c r="B17" s="1" t="n">
-        <v>0.561614954578717</v>
+        <v>0.56046189918867</v>
       </c>
     </row>
     <row r="18">
@@ -25147,7 +25147,7 @@
         <v>500</v>
       </c>
       <c r="B18" s="1" t="n">
-        <v>0.525786860392088</v>
+        <v>0.52665740669522</v>
       </c>
     </row>
     <row r="19">
@@ -25155,7 +25155,7 @@
         <v>501</v>
       </c>
       <c r="B19" s="1" t="n">
-        <v>0.530313709735418</v>
+        <v>0.531175274513231</v>
       </c>
     </row>
     <row r="20">
@@ -25163,7 +25163,7 @@
         <v>502</v>
       </c>
       <c r="B20" s="1" t="n">
-        <v>0.472540300670596</v>
+        <v>0.4734168561357</v>
       </c>
     </row>
     <row r="21">
@@ -25171,7 +25171,7 @@
         <v>503</v>
       </c>
       <c r="B21" s="1" t="n">
-        <v>0.384287779944996</v>
+        <v>0.384079025237481</v>
       </c>
     </row>
     <row r="22">
@@ -25179,7 +25179,7 @@
         <v>504</v>
       </c>
       <c r="B22" s="1" t="n">
-        <v>0.340115405485498</v>
+        <v>0.339490947848376</v>
       </c>
     </row>
     <row r="23">
@@ -25187,7 +25187,7 @@
         <v>505</v>
       </c>
       <c r="B23" s="1" t="n">
-        <v>0.31988896805625</v>
+        <v>0.319531354974</v>
       </c>
     </row>
     <row r="24">

</xml_diff>

<commit_message>
Corrida | SFE-ID | 2026-06-19 10:47:39.118039
</commit_message>
<xml_diff>
--- a/indicadores/SFE-ID_out.xlsx
+++ b/indicadores/SFE-ID_out.xlsx
@@ -113,13 +113,13 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">18/06/2026</t>
+    <t xml:space="preserve">19/06/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
   </si>
   <si>
-    <t xml:space="preserve">pcohan</t>
+    <t xml:space="preserve">fleiva</t>
   </si>
   <si>
     <t xml:space="preserve">fecha</t>
@@ -25261,4 +25261,237 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100C5B9F2161CEE1040BBC03CB11300495F" ma:contentTypeVersion="12" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="a7cec21613a3259523bdab11a1e26aca">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b5dd4176-d247-4204-85b8-921214f3ccea" xmlns:ns3="359b39ce-e1f9-4933-8424-33b611e6fdcd" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="68943c349d3a016936c8f8cb3335004b" ns2:_="" ns3:_="">
+    <xsd:import namespace="b5dd4176-d247-4204-85b8-921214f3ccea"/>
+    <xsd:import namespace="359b39ce-e1f9-4933-8424-33b611e6fdcd"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="b5dd4176-d247-4204-85b8-921214f3ccea" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="11" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Etiquetas de imagen" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="01529062-7a8b-4d76-943d-e0db5644ee6d" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="15" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="16" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="17" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="18" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="19" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="359b39ce-e1f9-4933-8424-33b611e6fdcd" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="14" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{c9b73259-0823-4f05-8927-4a40ee49fbe1}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="359b39ce-e1f9-4933-8424-33b611e6fdcd">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Tipo de contenido"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Título"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b5dd4176-d247-4204-85b8-921214f3ccea">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="359b39ce-e1f9-4933-8424-33b611e6fdcd" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CECC3124-C8DB-42A1-ABD5-ABD19718D613}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9CA32123-F03C-4555-A5A6-97D101ACECC6}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{19D3EAB3-E316-492E-BEBF-6CB7FD30DF94}"/>
 </file>
</xml_diff>

<commit_message>
Corrida | SFE-ID | 2026-06-24 09:16:53.363938
</commit_message>
<xml_diff>
--- a/indicadores/SFE-ID_out.xlsx
+++ b/indicadores/SFE-ID_out.xlsx
@@ -23,7 +23,7 @@
     <t xml:space="preserve">Título</t>
   </si>
   <si>
-    <t xml:space="preserve">Remuneraciones reales brutas de asegurados en ARTs</t>
+    <t xml:space="preserve">Remuneraciones brutas de asegurados en ARTs</t>
   </si>
   <si>
     <t xml:space="preserve">Unidad de medida</t>
@@ -113,7 +113,7 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">22/06/2026</t>
+    <t xml:space="preserve">24/06/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
@@ -2100,7 +2100,7 @@
       <c r="B11"/>
       <c r="C11"/>
       <c r="D11" t="n">
-        <v>0.617110624628424</v>
+        <v>0.613774016620658</v>
       </c>
       <c r="E11"/>
       <c r="F11"/>
@@ -2158,7 +2158,7 @@
       <c r="B15"/>
       <c r="C15"/>
       <c r="D15" t="n">
-        <v>0.380825523029284</v>
+        <v>0.376718543478656</v>
       </c>
       <c r="E15"/>
       <c r="F15"/>
@@ -2228,7 +2228,7 @@
       <c r="B20"/>
       <c r="C20"/>
       <c r="D20" t="n">
-        <v>0.759732661453156</v>
+        <v>0.755110999521041</v>
       </c>
       <c r="E20"/>
       <c r="F20"/>
@@ -2258,7 +2258,7 @@
       <c r="B22"/>
       <c r="C22"/>
       <c r="D22" t="n">
-        <v>0.000000079171049328658</v>
+        <v>0.0000000379540950916309</v>
       </c>
       <c r="E22"/>
       <c r="F22"/>
@@ -25089,7 +25089,7 @@
         <v>489</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>-0.00100889027184102</v>
+        <v>0.000104547807400108</v>
       </c>
     </row>
     <row r="6">
@@ -25097,7 +25097,7 @@
         <v>490</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>0.0315058543858523</v>
+        <v>0.034181074469872</v>
       </c>
     </row>
     <row r="7">
@@ -25105,7 +25105,7 @@
         <v>491</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>0.077025360381573</v>
+        <v>0.0775141723925324</v>
       </c>
     </row>
     <row r="8">
@@ -25113,7 +25113,7 @@
         <v>492</v>
       </c>
       <c r="B8" s="1" t="n">
-        <v>0.154675069647664</v>
+        <v>0.15190757437413</v>
       </c>
     </row>
     <row r="9">
@@ -25121,7 +25121,7 @@
         <v>493</v>
       </c>
       <c r="B9" s="1" t="n">
-        <v>0.213306856913311</v>
+        <v>0.21485947100407</v>
       </c>
     </row>
     <row r="10">
@@ -25129,7 +25129,7 @@
         <v>494</v>
       </c>
       <c r="B10" s="1" t="n">
-        <v>0.289218175326529</v>
+        <v>0.291393351626113</v>
       </c>
     </row>
     <row r="11">
@@ -25137,7 +25137,7 @@
         <v>495</v>
       </c>
       <c r="B11" s="1" t="n">
-        <v>0.377132390009974</v>
+        <v>0.377699271232895</v>
       </c>
     </row>
     <row r="12">
@@ -25145,7 +25145,7 @@
         <v>496</v>
       </c>
       <c r="B12" s="1" t="n">
-        <v>0.448482450591065</v>
+        <v>0.446223518652514</v>
       </c>
     </row>
     <row r="13">
@@ -25153,7 +25153,7 @@
         <v>497</v>
       </c>
       <c r="B13" s="1" t="n">
-        <v>0.516568343153864</v>
+        <v>0.510528975865804</v>
       </c>
     </row>
     <row r="14">
@@ -25161,7 +25161,7 @@
         <v>498</v>
       </c>
       <c r="B14" s="1" t="n">
-        <v>0.617110624628424</v>
+        <v>0.613774016620658</v>
       </c>
     </row>
     <row r="15">
@@ -25169,7 +25169,7 @@
         <v>499</v>
       </c>
       <c r="B15" s="1" t="n">
-        <v>0.594736898361042</v>
+        <v>0.592917883958775</v>
       </c>
     </row>
     <row r="16">
@@ -25177,7 +25177,7 @@
         <v>500</v>
       </c>
       <c r="B16" s="1" t="n">
-        <v>0.575910290347321</v>
+        <v>0.571820283774873</v>
       </c>
     </row>
     <row r="17">
@@ -25185,7 +25185,7 @@
         <v>501</v>
       </c>
       <c r="B17" s="1" t="n">
-        <v>0.557133540949434</v>
+        <v>0.557652800418566</v>
       </c>
     </row>
     <row r="18">
@@ -25193,7 +25193,7 @@
         <v>502</v>
       </c>
       <c r="B18" s="1" t="n">
-        <v>0.527378698846437</v>
+        <v>0.529020384181085</v>
       </c>
     </row>
     <row r="19">
@@ -25201,7 +25201,7 @@
         <v>503</v>
       </c>
       <c r="B19" s="1" t="n">
-        <v>0.534542985686977</v>
+        <v>0.533749056258202</v>
       </c>
     </row>
     <row r="20">
@@ -25209,7 +25209,7 @@
         <v>504</v>
       </c>
       <c r="B20" s="1" t="n">
-        <v>0.474361130752347</v>
+        <v>0.4749891682202</v>
       </c>
     </row>
     <row r="21">
@@ -25217,7 +25217,7 @@
         <v>505</v>
       </c>
       <c r="B21" s="1" t="n">
-        <v>0.38568068487037</v>
+        <v>0.386972158943423</v>
       </c>
     </row>
     <row r="22">
@@ -25225,7 +25225,7 @@
         <v>506</v>
       </c>
       <c r="B22" s="1" t="n">
-        <v>0.338469996593621</v>
+        <v>0.339757485570563</v>
       </c>
     </row>
     <row r="23">
@@ -25233,7 +25233,7 @@
         <v>507</v>
       </c>
       <c r="B23" s="1" t="n">
-        <v>0.314256703164556</v>
+        <v>0.313727776604649</v>
       </c>
     </row>
     <row r="24">

</xml_diff>

<commit_message>
Corrida | SFE-ID | 2026-07-14 12:17:21.539687
</commit_message>
<xml_diff>
--- a/indicadores/SFE-ID_out.xlsx
+++ b/indicadores/SFE-ID_out.xlsx
@@ -113,13 +113,13 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">24/06/2026</t>
+    <t xml:space="preserve">14/07/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
   </si>
   <si>
-    <t xml:space="preserve">fleiva</t>
+    <t xml:space="preserve">franco</t>
   </si>
   <si>
     <t xml:space="preserve">fecha</t>
@@ -2100,7 +2100,7 @@
       <c r="B11"/>
       <c r="C11"/>
       <c r="D11" t="n">
-        <v>0.613774016620658</v>
+        <v>0.60393637043565</v>
       </c>
       <c r="E11"/>
       <c r="F11"/>
@@ -2158,7 +2158,7 @@
       <c r="B15"/>
       <c r="C15"/>
       <c r="D15" t="n">
-        <v>0.376718543478656</v>
+        <v>0.364739139534987</v>
       </c>
       <c r="E15"/>
       <c r="F15"/>
@@ -2228,7 +2228,7 @@
       <c r="B20"/>
       <c r="C20"/>
       <c r="D20" t="n">
-        <v>0.755110999521041</v>
+        <v>0.859125929116967</v>
       </c>
       <c r="E20"/>
       <c r="F20"/>
@@ -2258,7 +2258,7 @@
       <c r="B22"/>
       <c r="C22"/>
       <c r="D22" t="n">
-        <v>0.0000000379540950916309</v>
+        <v>0.00000000730996159586486</v>
       </c>
       <c r="E22"/>
       <c r="F22"/>
@@ -25089,7 +25089,7 @@
         <v>489</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>0.000104547807400108</v>
+        <v>-0.0045930459527982</v>
       </c>
     </row>
     <row r="6">
@@ -25097,7 +25097,7 @@
         <v>490</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>0.034181074469872</v>
+        <v>0.0373903536564053</v>
       </c>
     </row>
     <row r="7">
@@ -25105,7 +25105,7 @@
         <v>491</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>0.0775141723925324</v>
+        <v>0.0824404625978667</v>
       </c>
     </row>
     <row r="8">
@@ -25113,7 +25113,7 @@
         <v>492</v>
       </c>
       <c r="B8" s="1" t="n">
-        <v>0.15190757437413</v>
+        <v>0.147717324140213</v>
       </c>
     </row>
     <row r="9">
@@ -25121,7 +25121,7 @@
         <v>493</v>
       </c>
       <c r="B9" s="1" t="n">
-        <v>0.21485947100407</v>
+        <v>0.217139986212436</v>
       </c>
     </row>
     <row r="10">
@@ -25129,7 +25129,7 @@
         <v>494</v>
       </c>
       <c r="B10" s="1" t="n">
-        <v>0.291393351626113</v>
+        <v>0.290671178085577</v>
       </c>
     </row>
     <row r="11">
@@ -25137,7 +25137,7 @@
         <v>495</v>
       </c>
       <c r="B11" s="1" t="n">
-        <v>0.377699271232895</v>
+        <v>0.380640689320811</v>
       </c>
     </row>
     <row r="12">
@@ -25145,7 +25145,7 @@
         <v>496</v>
       </c>
       <c r="B12" s="1" t="n">
-        <v>0.446223518652514</v>
+        <v>0.448470689384279</v>
       </c>
     </row>
     <row r="13">
@@ -25153,7 +25153,7 @@
         <v>497</v>
       </c>
       <c r="B13" s="1" t="n">
-        <v>0.510528975865804</v>
+        <v>0.527224003964839</v>
       </c>
     </row>
     <row r="14">
@@ -25161,7 +25161,7 @@
         <v>498</v>
       </c>
       <c r="B14" s="1" t="n">
-        <v>0.613774016620658</v>
+        <v>0.60393637043565</v>
       </c>
     </row>
     <row r="15">
@@ -25169,7 +25169,7 @@
         <v>499</v>
       </c>
       <c r="B15" s="1" t="n">
-        <v>0.592917883958775</v>
+        <v>0.601915696909055</v>
       </c>
     </row>
     <row r="16">
@@ -25177,7 +25177,7 @@
         <v>500</v>
       </c>
       <c r="B16" s="1" t="n">
-        <v>0.571820283774873</v>
+        <v>0.579303135611564</v>
       </c>
     </row>
     <row r="17">
@@ -25185,7 +25185,7 @@
         <v>501</v>
       </c>
       <c r="B17" s="1" t="n">
-        <v>0.557652800418566</v>
+        <v>0.551159159446635</v>
       </c>
     </row>
     <row r="18">
@@ -25193,7 +25193,7 @@
         <v>502</v>
       </c>
       <c r="B18" s="1" t="n">
-        <v>0.529020384181085</v>
+        <v>0.531718744372091</v>
       </c>
     </row>
     <row r="19">
@@ -25201,7 +25201,7 @@
         <v>503</v>
       </c>
       <c r="B19" s="1" t="n">
-        <v>0.533749056258202</v>
+        <v>0.532451818404494</v>
       </c>
     </row>
     <row r="20">
@@ -25209,7 +25209,7 @@
         <v>504</v>
       </c>
       <c r="B20" s="1" t="n">
-        <v>0.4749891682202</v>
+        <v>0.476397412486361</v>
       </c>
     </row>
     <row r="21">
@@ -25217,7 +25217,7 @@
         <v>505</v>
       </c>
       <c r="B21" s="1" t="n">
-        <v>0.386972158943423</v>
+        <v>0.391697019259597</v>
       </c>
     </row>
     <row r="22">
@@ -25225,7 +25225,7 @@
         <v>506</v>
       </c>
       <c r="B22" s="1" t="n">
-        <v>0.339757485570563</v>
+        <v>0.345417935543789</v>
       </c>
     </row>
     <row r="23">
@@ -25233,7 +25233,7 @@
         <v>507</v>
       </c>
       <c r="B23" s="1" t="n">
-        <v>0.313727776604649</v>
+        <v>0.309941576875246</v>
       </c>
     </row>
     <row r="24">
@@ -25261,4 +25261,237 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100C5B9F2161CEE1040BBC03CB11300495F" ma:contentTypeVersion="12" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="4b8b282811f2bcc11ff842570f663f4a">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b5dd4176-d247-4204-85b8-921214f3ccea" xmlns:ns3="359b39ce-e1f9-4933-8424-33b611e6fdcd" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="8b7f2ae8e4517a268e1f460c8f9cedce" ns2:_="" ns3:_="">
+    <xsd:import namespace="b5dd4176-d247-4204-85b8-921214f3ccea"/>
+    <xsd:import namespace="359b39ce-e1f9-4933-8424-33b611e6fdcd"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="b5dd4176-d247-4204-85b8-921214f3ccea" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="11" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="01529062-7a8b-4d76-943d-e0db5644ee6d" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="15" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="16" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="17" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="18" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="19" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="359b39ce-e1f9-4933-8424-33b611e6fdcd" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="14" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{c9b73259-0823-4f05-8927-4a40ee49fbe1}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="359b39ce-e1f9-4933-8424-33b611e6fdcd">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b5dd4176-d247-4204-85b8-921214f3ccea">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="359b39ce-e1f9-4933-8424-33b611e6fdcd" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D50F67CA-210A-4A64-9645-0DB59DF34098}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B88F1791-44EA-4DC9-B4CB-5D218C7BCA01}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D971691B-6869-403D-9EA0-62689D972A9B}"/>
 </file>
</xml_diff>

<commit_message>
Corrida | SFE-ID | 2026-07-14 12:24:05.295699
</commit_message>
<xml_diff>
--- a/indicadores/SFE-ID_out.xlsx
+++ b/indicadores/SFE-ID_out.xlsx
@@ -23,13 +23,13 @@
     <t xml:space="preserve">Título</t>
   </si>
   <si>
-    <t xml:space="preserve">Remuneraciones brutas de asegurados en ARTs</t>
+    <t xml:space="preserve">Remuneraciones reales brutas de asegurados en ARTs</t>
   </si>
   <si>
     <t xml:space="preserve">Unidad de medida</t>
   </si>
   <si>
-    <t xml:space="preserve">Miles de millones de pesos de 2025</t>
+    <t xml:space="preserve">Millones de pesos de 1993</t>
   </si>
   <si>
     <t xml:space="preserve">Ajuste estacional</t>
@@ -25261,237 +25261,4 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100C5B9F2161CEE1040BBC03CB11300495F" ma:contentTypeVersion="12" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="4b8b282811f2bcc11ff842570f663f4a">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b5dd4176-d247-4204-85b8-921214f3ccea" xmlns:ns3="359b39ce-e1f9-4933-8424-33b611e6fdcd" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="8b7f2ae8e4517a268e1f460c8f9cedce" ns2:_="" ns3:_="">
-    <xsd:import namespace="b5dd4176-d247-4204-85b8-921214f3ccea"/>
-    <xsd:import namespace="359b39ce-e1f9-4933-8424-33b611e6fdcd"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="b5dd4176-d247-4204-85b8-921214f3ccea" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="11" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="01529062-7a8b-4d76-943d-e0db5644ee6d" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="15" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="16" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="17" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="18" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="19" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="359b39ce-e1f9-4933-8424-33b611e6fdcd" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="TaxCatchAll" ma:index="14" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{c9b73259-0823-4f05-8927-4a40ee49fbe1}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="359b39ce-e1f9-4933-8424-33b611e6fdcd">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b5dd4176-d247-4204-85b8-921214f3ccea">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="359b39ce-e1f9-4933-8424-33b611e6fdcd" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D50F67CA-210A-4A64-9645-0DB59DF34098}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B88F1791-44EA-4DC9-B4CB-5D218C7BCA01}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D971691B-6869-403D-9EA0-62689D972A9B}"/>
 </file>
</xml_diff>

<commit_message>
Corrida | SFE-ID | 2026-07-14 12:25:28.683659
</commit_message>
<xml_diff>
--- a/indicadores/SFE-ID_out.xlsx
+++ b/indicadores/SFE-ID_out.xlsx
@@ -23,13 +23,13 @@
     <t xml:space="preserve">Título</t>
   </si>
   <si>
-    <t xml:space="preserve">Remuneraciones brutas de asegurados en ARTs</t>
+    <t xml:space="preserve">Remuneraciones reales brutas de asegurados en ARTs</t>
   </si>
   <si>
     <t xml:space="preserve">Unidad de medida</t>
   </si>
   <si>
-    <t xml:space="preserve">Miles de millones de pesos de 2025</t>
+    <t xml:space="preserve">Millones de pesos de 1993</t>
   </si>
   <si>
     <t xml:space="preserve">Ajuste estacional</t>
@@ -113,13 +113,13 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">24/06/2026</t>
+    <t xml:space="preserve">14/07/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
   </si>
   <si>
-    <t xml:space="preserve">fleiva</t>
+    <t xml:space="preserve">focampo</t>
   </si>
   <si>
     <t xml:space="preserve">fecha</t>
@@ -2100,7 +2100,7 @@
       <c r="B11"/>
       <c r="C11"/>
       <c r="D11" t="n">
-        <v>0.613774016620658</v>
+        <v>0.60393637043565</v>
       </c>
       <c r="E11"/>
       <c r="F11"/>
@@ -2158,7 +2158,7 @@
       <c r="B15"/>
       <c r="C15"/>
       <c r="D15" t="n">
-        <v>0.376718543478656</v>
+        <v>0.364739139534987</v>
       </c>
       <c r="E15"/>
       <c r="F15"/>
@@ -2228,7 +2228,7 @@
       <c r="B20"/>
       <c r="C20"/>
       <c r="D20" t="n">
-        <v>0.755110999521041</v>
+        <v>0.859125929116967</v>
       </c>
       <c r="E20"/>
       <c r="F20"/>
@@ -2258,7 +2258,7 @@
       <c r="B22"/>
       <c r="C22"/>
       <c r="D22" t="n">
-        <v>0.0000000379540950916309</v>
+        <v>0.00000000730996159586486</v>
       </c>
       <c r="E22"/>
       <c r="F22"/>
@@ -25089,7 +25089,7 @@
         <v>489</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>0.000104547807400108</v>
+        <v>-0.0045930459527982</v>
       </c>
     </row>
     <row r="6">
@@ -25097,7 +25097,7 @@
         <v>490</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>0.034181074469872</v>
+        <v>0.0373903536564053</v>
       </c>
     </row>
     <row r="7">
@@ -25105,7 +25105,7 @@
         <v>491</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>0.0775141723925324</v>
+        <v>0.0824404625978667</v>
       </c>
     </row>
     <row r="8">
@@ -25113,7 +25113,7 @@
         <v>492</v>
       </c>
       <c r="B8" s="1" t="n">
-        <v>0.15190757437413</v>
+        <v>0.147717324140213</v>
       </c>
     </row>
     <row r="9">
@@ -25121,7 +25121,7 @@
         <v>493</v>
       </c>
       <c r="B9" s="1" t="n">
-        <v>0.21485947100407</v>
+        <v>0.217139986212436</v>
       </c>
     </row>
     <row r="10">
@@ -25129,7 +25129,7 @@
         <v>494</v>
       </c>
       <c r="B10" s="1" t="n">
-        <v>0.291393351626113</v>
+        <v>0.290671178085577</v>
       </c>
     </row>
     <row r="11">
@@ -25137,7 +25137,7 @@
         <v>495</v>
       </c>
       <c r="B11" s="1" t="n">
-        <v>0.377699271232895</v>
+        <v>0.380640689320811</v>
       </c>
     </row>
     <row r="12">
@@ -25145,7 +25145,7 @@
         <v>496</v>
       </c>
       <c r="B12" s="1" t="n">
-        <v>0.446223518652514</v>
+        <v>0.448470689384279</v>
       </c>
     </row>
     <row r="13">
@@ -25153,7 +25153,7 @@
         <v>497</v>
       </c>
       <c r="B13" s="1" t="n">
-        <v>0.510528975865804</v>
+        <v>0.527224003964839</v>
       </c>
     </row>
     <row r="14">
@@ -25161,7 +25161,7 @@
         <v>498</v>
       </c>
       <c r="B14" s="1" t="n">
-        <v>0.613774016620658</v>
+        <v>0.60393637043565</v>
       </c>
     </row>
     <row r="15">
@@ -25169,7 +25169,7 @@
         <v>499</v>
       </c>
       <c r="B15" s="1" t="n">
-        <v>0.592917883958775</v>
+        <v>0.601915696909055</v>
       </c>
     </row>
     <row r="16">
@@ -25177,7 +25177,7 @@
         <v>500</v>
       </c>
       <c r="B16" s="1" t="n">
-        <v>0.571820283774873</v>
+        <v>0.579303135611564</v>
       </c>
     </row>
     <row r="17">
@@ -25185,7 +25185,7 @@
         <v>501</v>
       </c>
       <c r="B17" s="1" t="n">
-        <v>0.557652800418566</v>
+        <v>0.551159159446635</v>
       </c>
     </row>
     <row r="18">
@@ -25193,7 +25193,7 @@
         <v>502</v>
       </c>
       <c r="B18" s="1" t="n">
-        <v>0.529020384181085</v>
+        <v>0.531718744372091</v>
       </c>
     </row>
     <row r="19">
@@ -25201,7 +25201,7 @@
         <v>503</v>
       </c>
       <c r="B19" s="1" t="n">
-        <v>0.533749056258202</v>
+        <v>0.532451818404494</v>
       </c>
     </row>
     <row r="20">
@@ -25209,7 +25209,7 @@
         <v>504</v>
       </c>
       <c r="B20" s="1" t="n">
-        <v>0.4749891682202</v>
+        <v>0.476397412486361</v>
       </c>
     </row>
     <row r="21">
@@ -25217,7 +25217,7 @@
         <v>505</v>
       </c>
       <c r="B21" s="1" t="n">
-        <v>0.386972158943423</v>
+        <v>0.391697019259597</v>
       </c>
     </row>
     <row r="22">
@@ -25225,7 +25225,7 @@
         <v>506</v>
       </c>
       <c r="B22" s="1" t="n">
-        <v>0.339757485570563</v>
+        <v>0.345417935543789</v>
       </c>
     </row>
     <row r="23">
@@ -25233,7 +25233,7 @@
         <v>507</v>
       </c>
       <c r="B23" s="1" t="n">
-        <v>0.313727776604649</v>
+        <v>0.309941576875246</v>
       </c>
     </row>
     <row r="24">

</xml_diff>

<commit_message>
Corrida | SFE-ID | 2026-07-15 10:42:17.888013
</commit_message>
<xml_diff>
--- a/indicadores/SFE-ID_out.xlsx
+++ b/indicadores/SFE-ID_out.xlsx
@@ -26105,237 +26105,4 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100C5B9F2161CEE1040BBC03CB11300495F" ma:contentTypeVersion="12" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="4b8b282811f2bcc11ff842570f663f4a">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b5dd4176-d247-4204-85b8-921214f3ccea" xmlns:ns3="359b39ce-e1f9-4933-8424-33b611e6fdcd" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="8b7f2ae8e4517a268e1f460c8f9cedce" ns2:_="" ns3:_="">
-    <xsd:import namespace="b5dd4176-d247-4204-85b8-921214f3ccea"/>
-    <xsd:import namespace="359b39ce-e1f9-4933-8424-33b611e6fdcd"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="b5dd4176-d247-4204-85b8-921214f3ccea" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="11" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="01529062-7a8b-4d76-943d-e0db5644ee6d" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="15" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="16" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="17" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="18" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="19" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="359b39ce-e1f9-4933-8424-33b611e6fdcd" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="TaxCatchAll" ma:index="14" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{c9b73259-0823-4f05-8927-4a40ee49fbe1}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="359b39ce-e1f9-4933-8424-33b611e6fdcd">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b5dd4176-d247-4204-85b8-921214f3ccea">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="359b39ce-e1f9-4933-8424-33b611e6fdcd" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{28E349E6-7F99-41DC-9708-D7F92A198E35}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C6BE3FAE-B538-4241-A272-DA5E2935D045}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{82F9B29F-8225-4DBF-8921-B94FC75BDBE1}"/>
 </file>
</xml_diff>

<commit_message>
Corrida | SFE-ID | 2026-08-14 10:06:04.648394
</commit_message>
<xml_diff>
--- a/indicadores/SFE-ID_out.xlsx
+++ b/indicadores/SFE-ID_out.xlsx
@@ -24961,237 +24961,4 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100C5B9F2161CEE1040BBC03CB11300495F" ma:contentTypeVersion="12" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="a7cec21613a3259523bdab11a1e26aca">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b5dd4176-d247-4204-85b8-921214f3ccea" xmlns:ns3="359b39ce-e1f9-4933-8424-33b611e6fdcd" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="68943c349d3a016936c8f8cb3335004b" ns2:_="" ns3:_="">
-    <xsd:import namespace="b5dd4176-d247-4204-85b8-921214f3ccea"/>
-    <xsd:import namespace="359b39ce-e1f9-4933-8424-33b611e6fdcd"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="b5dd4176-d247-4204-85b8-921214f3ccea" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="11" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Etiquetas de imagen" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="01529062-7a8b-4d76-943d-e0db5644ee6d" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="15" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="16" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="17" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="18" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="19" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="359b39ce-e1f9-4933-8424-33b611e6fdcd" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="TaxCatchAll" ma:index="14" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{c9b73259-0823-4f05-8927-4a40ee49fbe1}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="359b39ce-e1f9-4933-8424-33b611e6fdcd">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Tipo de contenido"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Título"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b5dd4176-d247-4204-85b8-921214f3ccea">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="359b39ce-e1f9-4933-8424-33b611e6fdcd" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{68A8A1EF-0CC8-4E3A-B21E-87C656E5F9B4}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F30B3183-080C-4FFA-B415-156C2D3D015D}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8A074132-63DE-433D-AEEC-0AAEC712C9F8}"/>
 </file>
</xml_diff>

<commit_message>
Corrida | SFE-ID | 2026-09-02 08:20:20.305512
</commit_message>
<xml_diff>
--- a/indicadores/SFE-ID_out.xlsx
+++ b/indicadores/SFE-ID_out.xlsx
@@ -113,13 +113,13 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">14/08/2026</t>
+    <t xml:space="preserve">02/09/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
   </si>
   <si>
-    <t xml:space="preserve">vcorvalan</t>
+    <t xml:space="preserve">focampo</t>
   </si>
   <si>
     <t xml:space="preserve">fecha</t>
@@ -2082,7 +2082,7 @@
       <c r="B11"/>
       <c r="C11"/>
       <c r="D11" t="n">
-        <v>0.623143577986511</v>
+        <v>0.628050971118325</v>
       </c>
       <c r="E11"/>
       <c r="F11"/>
@@ -2140,7 +2140,7 @@
       <c r="B15"/>
       <c r="C15"/>
       <c r="D15" t="n">
-        <v>0.378334729699144</v>
+        <v>0.390702516936549</v>
       </c>
       <c r="E15"/>
       <c r="F15"/>
@@ -2210,7 +2210,7 @@
       <c r="B20"/>
       <c r="C20"/>
       <c r="D20" t="n">
-        <v>0.417191220409216</v>
+        <v>0.555311060554717</v>
       </c>
       <c r="E20"/>
       <c r="F20"/>
@@ -2240,7 +2240,7 @@
       <c r="B22"/>
       <c r="C22"/>
       <c r="D22" t="n">
-        <v>0.000000015959859669501</v>
+        <v>0.0000000183041455600604</v>
       </c>
       <c r="E22"/>
       <c r="F22"/>
@@ -24789,7 +24789,7 @@
         <v>483</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>-0.0221566498333309</v>
+        <v>-0.0156383377844672</v>
       </c>
     </row>
     <row r="6">
@@ -24797,7 +24797,7 @@
         <v>484</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>0.0241100921887178</v>
+        <v>0.0299827436558771</v>
       </c>
     </row>
     <row r="7">
@@ -24805,7 +24805,7 @@
         <v>485</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>0.0690638508443012</v>
+        <v>0.0764703918057814</v>
       </c>
     </row>
     <row r="8">
@@ -24813,7 +24813,7 @@
         <v>486</v>
       </c>
       <c r="B8" s="1" t="n">
-        <v>0.144682714373852</v>
+        <v>0.149714874231264</v>
       </c>
     </row>
     <row r="9">
@@ -24821,7 +24821,7 @@
         <v>487</v>
       </c>
       <c r="B9" s="1" t="n">
-        <v>0.212976119495992</v>
+        <v>0.218326197740142</v>
       </c>
     </row>
     <row r="10">
@@ -24829,7 +24829,7 @@
         <v>488</v>
       </c>
       <c r="B10" s="1" t="n">
-        <v>0.286236775074382</v>
+        <v>0.29554118789791</v>
       </c>
     </row>
     <row r="11">
@@ -24837,7 +24837,7 @@
         <v>489</v>
       </c>
       <c r="B11" s="1" t="n">
-        <v>0.376279104595764</v>
+        <v>0.381051865899579</v>
       </c>
     </row>
     <row r="12">
@@ -24845,7 +24845,7 @@
         <v>490</v>
       </c>
       <c r="B12" s="1" t="n">
-        <v>0.449958799661195</v>
+        <v>0.451616348534244</v>
       </c>
     </row>
     <row r="13">
@@ -24853,7 +24853,7 @@
         <v>491</v>
       </c>
       <c r="B13" s="1" t="n">
-        <v>0.538278152308813</v>
+        <v>0.547634113516833</v>
       </c>
     </row>
     <row r="14">
@@ -24861,7 +24861,7 @@
         <v>492</v>
       </c>
       <c r="B14" s="1" t="n">
-        <v>0.615089204668024</v>
+        <v>0.625062010473</v>
       </c>
     </row>
     <row r="15">
@@ -24869,7 +24869,7 @@
         <v>493</v>
       </c>
       <c r="B15" s="1" t="n">
-        <v>0.623143577986511</v>
+        <v>0.628050971118325</v>
       </c>
     </row>
     <row r="16">
@@ -24877,7 +24877,7 @@
         <v>494</v>
       </c>
       <c r="B16" s="1" t="n">
-        <v>0.593089631484677</v>
+        <v>0.601303233947716</v>
       </c>
     </row>
     <row r="17">
@@ -24885,7 +24885,7 @@
         <v>495</v>
       </c>
       <c r="B17" s="1" t="n">
-        <v>0.580552252095618</v>
+        <v>0.587791211827087</v>
       </c>
     </row>
     <row r="18">
@@ -24893,7 +24893,7 @@
         <v>496</v>
       </c>
       <c r="B18" s="1" t="n">
-        <v>0.557303137025625</v>
+        <v>0.558386334115931</v>
       </c>
     </row>
     <row r="19">
@@ -24901,7 +24901,7 @@
         <v>497</v>
       </c>
       <c r="B19" s="1" t="n">
-        <v>0.55356852211296</v>
+        <v>0.553084080821669</v>
       </c>
     </row>
     <row r="20">
@@ -24909,7 +24909,7 @@
         <v>498</v>
       </c>
       <c r="B20" s="1" t="n">
-        <v>0.497039055850604</v>
+        <v>0.498383455196921</v>
       </c>
     </row>
     <row r="21">
@@ -24917,7 +24917,7 @@
         <v>499</v>
       </c>
       <c r="B21" s="1" t="n">
-        <v>0.41312117397884</v>
+        <v>0.418162009382583</v>
       </c>
     </row>
     <row r="22">
@@ -24925,7 +24925,7 @@
         <v>500</v>
       </c>
       <c r="B22" s="1" t="n">
-        <v>0.356455644674103</v>
+        <v>0.365539583278729</v>
       </c>
     </row>
     <row r="23">
@@ -24933,7 +24933,7 @@
         <v>501</v>
       </c>
       <c r="B23" s="1" t="n">
-        <v>0.321011720188394</v>
+        <v>0.32878427301448</v>
       </c>
     </row>
     <row r="24">
@@ -24961,4 +24961,237 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100C5B9F2161CEE1040BBC03CB11300495F" ma:contentTypeVersion="12" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="a7cec21613a3259523bdab11a1e26aca">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b5dd4176-d247-4204-85b8-921214f3ccea" xmlns:ns3="359b39ce-e1f9-4933-8424-33b611e6fdcd" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="68943c349d3a016936c8f8cb3335004b" ns2:_="" ns3:_="">
+    <xsd:import namespace="b5dd4176-d247-4204-85b8-921214f3ccea"/>
+    <xsd:import namespace="359b39ce-e1f9-4933-8424-33b611e6fdcd"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="b5dd4176-d247-4204-85b8-921214f3ccea" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="11" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Etiquetas de imagen" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="01529062-7a8b-4d76-943d-e0db5644ee6d" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="15" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="16" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="17" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="18" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="19" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="359b39ce-e1f9-4933-8424-33b611e6fdcd" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="14" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{c9b73259-0823-4f05-8927-4a40ee49fbe1}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="359b39ce-e1f9-4933-8424-33b611e6fdcd">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Tipo de contenido"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Título"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b5dd4176-d247-4204-85b8-921214f3ccea">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="359b39ce-e1f9-4933-8424-33b611e6fdcd" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{56CAFB24-DB2D-4766-92DE-404F5A5014B8}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4D13066A-E92B-4F98-A646-A5FD4E68AF6C}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7DAD33C3-333B-4039-AC03-DFF351439C63}"/>
 </file>
</xml_diff>

<commit_message>
Corrida | SFE-ID | 2026-09-11 08:42:34.07229
</commit_message>
<xml_diff>
--- a/indicadores/SFE-ID_out.xlsx
+++ b/indicadores/SFE-ID_out.xlsx
@@ -113,7 +113,7 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">04/09/2026</t>
+    <t xml:space="preserve">11/09/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
@@ -2110,7 +2110,7 @@
       <c r="B11"/>
       <c r="C11"/>
       <c r="D11" t="n">
-        <v>0.609981087317274</v>
+        <v>0.60985129405743</v>
       </c>
       <c r="E11"/>
       <c r="F11"/>
@@ -2168,7 +2168,7 @@
       <c r="B15"/>
       <c r="C15"/>
       <c r="D15" t="n">
-        <v>0.372076926884763</v>
+        <v>0.371918600863522</v>
       </c>
       <c r="E15"/>
       <c r="F15"/>
@@ -2238,7 +2238,7 @@
       <c r="B20"/>
       <c r="C20"/>
       <c r="D20" t="n">
-        <v>0.75195831347292</v>
+        <v>0.747384519613737</v>
       </c>
       <c r="E20"/>
       <c r="F20"/>
@@ -2268,7 +2268,7 @@
       <c r="B22"/>
       <c r="C22"/>
       <c r="D22" t="n">
-        <v>0.000000000772089612758351</v>
+        <v>0.000000000755405543628716</v>
       </c>
       <c r="E22"/>
       <c r="F22"/>
@@ -26005,7 +26005,7 @@
         <v>491</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>-0.0107991654422695</v>
+        <v>-0.0106687978211678</v>
       </c>
     </row>
     <row r="6">
@@ -26013,7 +26013,7 @@
         <v>492</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>0.0288771477766835</v>
+        <v>0.0287914747685185</v>
       </c>
     </row>
     <row r="7">
@@ -26021,7 +26021,7 @@
         <v>493</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>0.0734482837368624</v>
+        <v>0.0736522664590632</v>
       </c>
     </row>
     <row r="8">
@@ -26029,7 +26029,7 @@
         <v>494</v>
       </c>
       <c r="B8" s="1" t="n">
-        <v>0.143202985044223</v>
+        <v>0.143401692143215</v>
       </c>
     </row>
     <row r="9">
@@ -26037,7 +26037,7 @@
         <v>495</v>
       </c>
       <c r="B9" s="1" t="n">
-        <v>0.209413557888027</v>
+        <v>0.209181930016259</v>
       </c>
     </row>
     <row r="10">
@@ -26045,7 +26045,7 @@
         <v>496</v>
       </c>
       <c r="B10" s="1" t="n">
-        <v>0.276330356241573</v>
+        <v>0.276514017967997</v>
       </c>
     </row>
     <row r="11">
@@ -26053,7 +26053,7 @@
         <v>497</v>
       </c>
       <c r="B11" s="1" t="n">
-        <v>0.353867989331048</v>
+        <v>0.354453647686085</v>
       </c>
     </row>
     <row r="12">
@@ -26061,7 +26061,7 @@
         <v>498</v>
       </c>
       <c r="B12" s="1" t="n">
-        <v>0.431294302066894</v>
+        <v>0.431357399371021</v>
       </c>
     </row>
     <row r="13">
@@ -26069,7 +26069,7 @@
         <v>499</v>
       </c>
       <c r="B13" s="1" t="n">
-        <v>0.517928455668221</v>
+        <v>0.517694602182123</v>
       </c>
     </row>
     <row r="14">
@@ -26077,7 +26077,7 @@
         <v>500</v>
       </c>
       <c r="B14" s="1" t="n">
-        <v>0.609981087317274</v>
+        <v>0.60985129405743</v>
       </c>
     </row>
     <row r="15">
@@ -26085,7 +26085,7 @@
         <v>501</v>
       </c>
       <c r="B15" s="1" t="n">
-        <v>0.60517385427987</v>
+        <v>0.605006257371677</v>
       </c>
     </row>
     <row r="16">
@@ -26093,7 +26093,7 @@
         <v>502</v>
       </c>
       <c r="B16" s="1" t="n">
-        <v>0.57697001490974</v>
+        <v>0.57656627377129</v>
       </c>
     </row>
     <row r="17">
@@ -26101,7 +26101,7 @@
         <v>503</v>
       </c>
       <c r="B17" s="1" t="n">
-        <v>0.560966302028843</v>
+        <v>0.560151616948722</v>
       </c>
     </row>
     <row r="18">
@@ -26109,7 +26109,7 @@
         <v>504</v>
       </c>
       <c r="B18" s="1" t="n">
-        <v>0.535661882738633</v>
+        <v>0.535052172000342</v>
       </c>
     </row>
     <row r="19">
@@ -26117,7 +26117,7 @@
         <v>505</v>
       </c>
       <c r="B19" s="1" t="n">
-        <v>0.527298960213111</v>
+        <v>0.526998629936701</v>
       </c>
     </row>
     <row r="20">
@@ -26125,7 +26125,7 @@
         <v>506</v>
       </c>
       <c r="B20" s="1" t="n">
-        <v>0.479851909999592</v>
+        <v>0.479644030935983</v>
       </c>
     </row>
     <row r="21">
@@ -26133,7 +26133,7 @@
         <v>507</v>
       </c>
       <c r="B21" s="1" t="n">
-        <v>0.391521670403578</v>
+        <v>0.39171315512839</v>
       </c>
     </row>
     <row r="22">
@@ -26141,7 +26141,7 @@
         <v>508</v>
       </c>
       <c r="B22" s="1" t="n">
-        <v>0.344905193907737</v>
+        <v>0.34502612230553</v>
       </c>
     </row>
     <row r="23">
@@ -26149,7 +26149,7 @@
         <v>509</v>
       </c>
       <c r="B23" s="1" t="n">
-        <v>0.320431574422312</v>
+        <v>0.320404550607726</v>
       </c>
     </row>
     <row r="24">

</xml_diff>